<commit_message>
Add CAP776 Minor Project 1
</commit_message>
<xml_diff>
--- a/Downloads/daily activty log/12614864.xlsx
+++ b/Downloads/daily activty log/12614864.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\daily activty log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1C3DDD-A24A-403F-8AB6-E80BCBB5EAD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E594B6-1A4E-44C1-83EB-D5E6868DCDEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="95">
   <si>
     <t>My Data, My Code — Daily Log</t>
   </si>
@@ -309,6 +309,15 @@
   <si>
     <t>Stayed at home again. Did some study and completed a few work tasks.</t>
   </si>
+  <si>
+    <t>College was closed. Studied for a few hours and worked on my project.</t>
+  </si>
+  <si>
+    <t>College was closed again. Focused on study and finished some pending work.</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
 </sst>
 </file>
 
@@ -469,7 +478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -510,27 +519,12 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1014,74 +1008,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="19"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="20">
         <v>12614864</v>
       </c>
-      <c r="G2" s="19"/>
+      <c r="G2" s="21"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="19"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="21"/>
       <c r="E3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="21"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
     </row>
     <row r="5" spans="1:14" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -3474,268 +3468,312 @@
       </c>
     </row>
     <row r="57" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="24">
+      <c r="A57" s="8">
         <v>46291</v>
       </c>
-      <c r="B57" s="25">
+      <c r="B57" s="9">
         <v>480</v>
       </c>
-      <c r="C57" s="25">
+      <c r="C57" s="9">
         <v>30</v>
       </c>
-      <c r="D57" s="25">
+      <c r="D57" s="9">
         <v>180</v>
       </c>
-      <c r="E57" s="25">
+      <c r="E57" s="9">
         <v>150</v>
       </c>
-      <c r="F57" s="25">
+      <c r="F57" s="9">
         <v>0</v>
       </c>
-      <c r="G57" s="25">
+      <c r="G57" s="9">
         <v>0</v>
       </c>
-      <c r="H57" s="25">
+      <c r="H57" s="9">
         <v>120</v>
       </c>
-      <c r="I57" s="26">
+      <c r="I57" s="10">
         <v>960</v>
       </c>
-      <c r="J57" s="26">
+      <c r="J57" s="10">
         <v>480</v>
       </c>
-      <c r="K57" s="27" t="s">
+      <c r="K57" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="L57" s="27" t="s">
+      <c r="L57" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="M57" s="27" t="s">
+      <c r="M57" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="N57" s="28" t="s">
+      <c r="N57" s="12" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="58" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A58" s="24">
+      <c r="A58" s="8">
         <v>46292</v>
       </c>
-      <c r="B58" s="25">
+      <c r="B58" s="9">
         <v>510</v>
       </c>
-      <c r="C58" s="25">
+      <c r="C58" s="9">
         <v>0</v>
       </c>
-      <c r="D58" s="25">
+      <c r="D58" s="9">
         <v>150</v>
       </c>
-      <c r="E58" s="25">
+      <c r="E58" s="9">
         <v>120</v>
       </c>
-      <c r="F58" s="25">
+      <c r="F58" s="9">
         <v>0</v>
       </c>
-      <c r="G58" s="25">
+      <c r="G58" s="9">
         <v>0</v>
       </c>
-      <c r="H58" s="25">
+      <c r="H58" s="9">
         <v>180</v>
       </c>
-      <c r="I58" s="26">
+      <c r="I58" s="10">
         <v>960</v>
       </c>
-      <c r="J58" s="26">
+      <c r="J58" s="10">
         <v>480</v>
       </c>
-      <c r="K58" s="27" t="s">
+      <c r="K58" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="L58" s="27" t="s">
+      <c r="L58" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="M58" s="27" t="s">
+      <c r="M58" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="N58" s="28" t="s">
+      <c r="N58" s="12" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="59" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A59" s="24">
+      <c r="A59" s="8">
         <v>46293</v>
       </c>
-      <c r="B59" s="25">
+      <c r="B59" s="9">
         <v>450</v>
       </c>
-      <c r="C59" s="25">
+      <c r="C59" s="9">
         <v>30</v>
       </c>
-      <c r="D59" s="25">
+      <c r="D59" s="9">
         <v>210</v>
       </c>
-      <c r="E59" s="25">
+      <c r="E59" s="9">
         <v>180</v>
       </c>
-      <c r="F59" s="25">
+      <c r="F59" s="9">
         <v>0</v>
       </c>
-      <c r="G59" s="25">
+      <c r="G59" s="9">
         <v>0</v>
       </c>
-      <c r="H59" s="25">
+      <c r="H59" s="9">
         <v>120</v>
       </c>
-      <c r="I59" s="26">
+      <c r="I59" s="10">
         <v>990</v>
       </c>
-      <c r="J59" s="26">
+      <c r="J59" s="10">
         <v>450</v>
       </c>
-      <c r="K59" s="27" t="s">
+      <c r="K59" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="L59" s="27" t="s">
+      <c r="L59" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="M59" s="27" t="s">
+      <c r="M59" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="N59" s="28" t="s">
+      <c r="N59" s="12" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="60" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="24">
+      <c r="A60" s="8">
         <v>46294</v>
       </c>
-      <c r="B60" s="25">
+      <c r="B60" s="9">
         <v>420</v>
       </c>
-      <c r="C60" s="25">
+      <c r="C60" s="9">
         <v>0</v>
       </c>
-      <c r="D60" s="25">
+      <c r="D60" s="9">
         <v>180</v>
       </c>
-      <c r="E60" s="25">
+      <c r="E60" s="9">
         <v>240</v>
       </c>
-      <c r="F60" s="25">
+      <c r="F60" s="9">
         <v>0</v>
       </c>
-      <c r="G60" s="25">
+      <c r="G60" s="9">
         <v>0</v>
       </c>
-      <c r="H60" s="25">
+      <c r="H60" s="9">
         <v>150</v>
       </c>
-      <c r="I60" s="26">
+      <c r="I60" s="10">
         <v>990</v>
       </c>
-      <c r="J60" s="26">
+      <c r="J60" s="10">
         <v>450</v>
       </c>
-      <c r="K60" s="27" t="s">
+      <c r="K60" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="L60" s="27" t="s">
+      <c r="L60" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="M60" s="27" t="s">
+      <c r="M60" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="N60" s="28" t="s">
+      <c r="N60" s="12" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="61" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A61" s="24">
+      <c r="A61" s="8">
         <v>46295</v>
       </c>
-      <c r="B61" s="25">
+      <c r="B61" s="9">
         <v>480</v>
       </c>
-      <c r="C61" s="25">
+      <c r="C61" s="9">
         <v>30</v>
       </c>
-      <c r="D61" s="25">
+      <c r="D61" s="9">
         <v>150</v>
       </c>
-      <c r="E61" s="25">
+      <c r="E61" s="9">
         <v>180</v>
       </c>
-      <c r="F61" s="25">
+      <c r="F61" s="9">
         <v>0</v>
       </c>
-      <c r="G61" s="25">
+      <c r="G61" s="9">
         <v>0</v>
       </c>
-      <c r="H61" s="25">
+      <c r="H61" s="9">
         <v>150</v>
       </c>
-      <c r="I61" s="26">
+      <c r="I61" s="10">
         <v>990</v>
       </c>
-      <c r="J61" s="26">
+      <c r="J61" s="10">
         <v>450</v>
       </c>
-      <c r="K61" s="27" t="s">
+      <c r="K61" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="L61" s="27" t="s">
+      <c r="L61" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="M61" s="27" t="s">
+      <c r="M61" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="N61" s="28" t="s">
+      <c r="N61" s="12" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="8"/>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="9"/>
-      <c r="F62" s="9"/>
-      <c r="G62" s="9"/>
-      <c r="H62" s="9"/>
-      <c r="I62" s="10" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J62" s="10" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K62" s="11"/>
-      <c r="L62" s="11"/>
-      <c r="M62" s="11"/>
-      <c r="N62" s="12"/>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="8"/>
-      <c r="B63" s="9"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="9"/>
-      <c r="F63" s="9"/>
-      <c r="G63" s="9"/>
-      <c r="H63" s="9"/>
-      <c r="I63" s="10" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J63" s="10" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K63" s="11"/>
-      <c r="L63" s="11"/>
-      <c r="M63" s="11"/>
-      <c r="N63" s="12"/>
+    <row r="62" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A62" s="8">
+        <v>46296</v>
+      </c>
+      <c r="B62" s="9">
+        <v>450</v>
+      </c>
+      <c r="C62" s="9">
+        <v>30</v>
+      </c>
+      <c r="D62" s="9">
+        <v>180</v>
+      </c>
+      <c r="E62" s="9">
+        <v>150</v>
+      </c>
+      <c r="F62" s="9">
+        <v>0</v>
+      </c>
+      <c r="G62" s="9">
+        <v>0</v>
+      </c>
+      <c r="H62" s="9">
+        <v>120</v>
+      </c>
+      <c r="I62" s="10">
+        <v>930</v>
+      </c>
+      <c r="J62" s="10">
+        <v>510</v>
+      </c>
+      <c r="K62" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L62" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="M62" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N62" s="12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A63" s="8">
+        <v>46297</v>
+      </c>
+      <c r="B63" s="9">
+        <v>480</v>
+      </c>
+      <c r="C63" s="9">
+        <v>40</v>
+      </c>
+      <c r="D63" s="9">
+        <v>150</v>
+      </c>
+      <c r="E63" s="9">
+        <v>210</v>
+      </c>
+      <c r="F63" s="9">
+        <v>0</v>
+      </c>
+      <c r="G63" s="9">
+        <v>0</v>
+      </c>
+      <c r="H63" s="9">
+        <v>150</v>
+      </c>
+      <c r="I63" s="10">
+        <v>1030</v>
+      </c>
+      <c r="J63" s="10">
+        <v>410</v>
+      </c>
+      <c r="K63" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="L63" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="M63" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N63" s="12" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="8"/>
@@ -3762,7 +3800,9 @@
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" s="8"/>
       <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
+      <c r="C65" s="9" t="s">
+        <v>94</v>
+      </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9"/>
       <c r="F65" s="9"/>
@@ -10919,11 +10959,11 @@
       <c r="G390" s="9"/>
       <c r="H390" s="9"/>
       <c r="I390" s="10" t="str">
-        <f t="shared" ref="I390:I453" si="12">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I401" si="12">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="10" t="str">
-        <f t="shared" ref="J390:J453" si="13">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="13">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="11"/>

</xml_diff>